<commit_message>
Corrections des erreurs de hiérarchie
</commit_message>
<xml_diff>
--- a/tools/excel/PASSI/PASSI.xlsx
+++ b/tools/excel/PASSI/PASSI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cintamaya-my.sharepoint.com/personal/arthur_lafont_cintamaya_com/Documents/02.Cinta/Ciso import tool/ciso-assistant-community/tools/excel/PASSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="84" documentId="13_ncr:1_{C69144C6-7723-45D0-AD2A-8B323A6D48CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{903E983D-73F8-4A5E-8D2C-BCD5F06E26AA}"/>
+  <xr:revisionPtr revIDLastSave="90" documentId="13_ncr:1_{C69144C6-7723-45D0-AD2A-8B323A6D48CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{827C76A5-B2E3-40AB-B035-53C2628F1EEC}"/>
   <bookViews>
-    <workbookView xWindow="14205" yWindow="-16425" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14205" yWindow="-16425" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="library_meta" sheetId="2" r:id="rId1"/>
@@ -299,12 +299,6 @@
     <t>V.1.d</t>
   </si>
   <si>
-    <t>Les auditeurs et responsables d’équipe doivent maîtriser les bonnes pratiques et la méthodologie d’audit décrites dans la norme  ISO/IEC 1901.</t>
-  </si>
-  <si>
-    <t>Les auditeurs doivent posséder les qualités personnelles décrites au chapitre « 7.2.2 Comportements personnels » de la norme  ISO/IEC 1901.</t>
-  </si>
-  <si>
     <t>Les auditeurs et responsables d’équipe doivent disposer de qualités rédactionnelles et de synthèse, et savoir restituer les informations pertinentes et adaptées aux profils de leurs interlocuteurs (direction, services techniques, responsables métier et sécurité, etc.).</t>
   </si>
   <si>
@@ -612,12 +606,6 @@
   </si>
   <si>
     <t>VI.3</t>
-  </si>
-  <si>
-    <t>préciser que le prestataire peut incorporer dans l’équipe d’audit un ou plusieurs experts pour participer à la réalisation de certaines activités d’audit lorsque ces dernières requièrent des connaissances ou des compétences spécifiques dont les auditeurs ne disposent pas sous réserve que : 
-i. il existe une un cadre contractuel entre le prestataire et les experts ;
-ii. le recours aux experts est accepté par le commanditaire ;
-iii. les experts sont dûment encadrés par le responsable d’équipe.</t>
   </si>
   <si>
     <t>préciser que le prestataire peut sous-traiter tout ou partie des activités d’audit à un prestataire sous-traitant sous réserve que : 
@@ -1272,9 +1260,6 @@
   </si>
   <si>
     <t>Le prestataire doit s’assurer, avant le début de chaque prestation, que les membres de l'équipe, disposent des connaissances et compétences associées à leurs activités conformément à l’Annexe 2.</t>
-  </si>
-  <si>
-    <t>Il est recommandé que le prestataire mette en œuvre la démarche décrite dans le guide pour homologuer son d’information.</t>
   </si>
   <si>
     <t>Le prestataire doit disposer d’un système d’information hors ligne afin de conserver l’ensemble des informations et supports relatifs à la prestation pour lesquels il a reçu une autorisation de conservation du commanditaire.</t>
@@ -1427,6 +1412,21 @@
   </si>
   <si>
     <t>PASSI Framework 2.2</t>
+  </si>
+  <si>
+    <t>Il est recommandé que le prestataire mette en œuvre la démarche décrite dans le guide pour homologuer son système d’information.</t>
+  </si>
+  <si>
+    <t>Les auditeurs et responsables d’équipe doivent maîtriser les bonnes pratiques et la méthodologie d’audit décrites dans la norme  ISO 1901.</t>
+  </si>
+  <si>
+    <t>Les auditeurs doivent posséder les qualités personnelles décrites au chapitre « 7.2.2 Comportements personnels » de la norme  ISO 1901.</t>
+  </si>
+  <si>
+    <t>préciser que le prestataire peut incorporer dans l’équipe d’audit un ou plusieurs experts pour participer à la réalisation de certaines activités d’audit lorsque ces dernières requièrent des connaissances ou des compétences spécifiques dont les auditeurs ne disposent pas sous réserve que : 
+i. il existe un cadre contractuel entre le prestataire et les experts ;
+ii. le recours aux experts est accepté par le commanditaire ;
+iii. les experts sont dûment encadrés par le responsable d’équipe.</t>
   </si>
 </sst>
 </file>
@@ -1825,23 +1825,23 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>419</v>
+        <v>415</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>432</v>
+        <v>428</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>421</v>
+        <v>417</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
@@ -1849,7 +1849,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>422</v>
+        <v>418</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>8</v>
@@ -1860,7 +1860,7 @@
         <v>4</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>435</v>
+        <v>431</v>
       </c>
     </row>
     <row r="6" spans="1:2" x14ac:dyDescent="0.3">
@@ -1868,7 +1868,7 @@
         <v>2</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="57.6" x14ac:dyDescent="0.3">
@@ -1876,28 +1876,28 @@
         <v>5</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>423</v>
+        <v>419</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>424</v>
+        <v>420</v>
       </c>
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>425</v>
+        <v>421</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>431</v>
+        <v>427</v>
       </c>
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>426</v>
+        <v>422</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>11</v>
@@ -1920,26 +1920,26 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s">
-        <v>427</v>
+        <v>423</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>428</v>
+        <v>424</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>433</v>
+        <v>429</v>
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>420</v>
+        <v>416</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
@@ -1963,15 +1963,15 @@
         <v>5</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>430</v>
+        <v>426</v>
       </c>
       <c r="B7" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>
@@ -2019,10 +2019,10 @@
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
@@ -2030,10 +2030,10 @@
         <v>2</v>
       </c>
       <c r="D3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
@@ -2177,10 +2177,10 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E12" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="13" spans="1:7" ht="28.8" x14ac:dyDescent="0.3">
@@ -2214,7 +2214,7 @@
         <v>26</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
     </row>
     <row r="15" spans="1:7" ht="57.6" x14ac:dyDescent="0.3">
@@ -2324,10 +2324,10 @@
         <v>2</v>
       </c>
       <c r="D21" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E21" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
@@ -2480,7 +2480,7 @@
         <v>52</v>
       </c>
       <c r="F30" s="3" t="s">
-        <v>400</v>
+        <v>432</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
@@ -2616,7 +2616,7 @@
         <v>60</v>
       </c>
       <c r="F38" s="3" t="s">
-        <v>401</v>
+        <v>397</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
@@ -2624,10 +2624,10 @@
         <v>1</v>
       </c>
       <c r="D39" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="E39" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
@@ -2635,10 +2635,10 @@
         <v>2</v>
       </c>
       <c r="D40" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="E40" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
     </row>
     <row r="41" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2655,7 +2655,7 @@
         <v>81</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>85</v>
+        <v>433</v>
       </c>
     </row>
     <row r="42" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2672,7 +2672,7 @@
         <v>82</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>86</v>
+        <v>434</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2689,7 +2689,7 @@
         <v>83</v>
       </c>
       <c r="F43" s="3" t="s">
-        <v>402</v>
+        <v>398</v>
       </c>
     </row>
     <row r="44" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2706,7 +2706,7 @@
         <v>84</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
@@ -2714,10 +2714,10 @@
         <v>2</v>
       </c>
       <c r="D45" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="E45" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
@@ -2731,10 +2731,10 @@
         <v>71</v>
       </c>
       <c r="D46" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F46" s="3" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
@@ -2748,10 +2748,10 @@
         <v>71</v>
       </c>
       <c r="D47" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="F47" s="3" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2765,10 +2765,10 @@
         <v>71</v>
       </c>
       <c r="D48" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
@@ -2776,10 +2776,10 @@
         <v>2</v>
       </c>
       <c r="D49" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="E49" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
@@ -2793,10 +2793,10 @@
         <v>71</v>
       </c>
       <c r="D50" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2810,10 +2810,10 @@
         <v>71</v>
       </c>
       <c r="D51" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
@@ -2821,10 +2821,10 @@
         <v>2</v>
       </c>
       <c r="D52" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="E52" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
@@ -2838,10 +2838,10 @@
         <v>71</v>
       </c>
       <c r="D53" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="F53" s="3" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
@@ -2855,10 +2855,10 @@
         <v>71</v>
       </c>
       <c r="D54" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="F54" s="3" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
@@ -2866,10 +2866,10 @@
         <v>1</v>
       </c>
       <c r="D55" t="s">
+        <v>182</v>
+      </c>
+      <c r="E55" t="s">
         <v>184</v>
-      </c>
-      <c r="E55" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
@@ -2877,10 +2877,10 @@
         <v>2</v>
       </c>
       <c r="D56" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="E56" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -2894,10 +2894,10 @@
         <v>71</v>
       </c>
       <c r="D57" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F57" s="3" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2911,10 +2911,10 @@
         <v>71</v>
       </c>
       <c r="D58" t="s">
+        <v>101</v>
+      </c>
+      <c r="F58" s="3" t="s">
         <v>103</v>
-      </c>
-      <c r="F58" s="3" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2928,10 +2928,10 @@
         <v>71</v>
       </c>
       <c r="D59" t="s">
+        <v>102</v>
+      </c>
+      <c r="F59" s="3" t="s">
         <v>104</v>
-      </c>
-      <c r="F59" s="3" t="s">
-        <v>106</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
@@ -2939,10 +2939,10 @@
         <v>2</v>
       </c>
       <c r="D60" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="E60" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
@@ -2956,10 +2956,10 @@
         <v>71</v>
       </c>
       <c r="D61" t="s">
+        <v>105</v>
+      </c>
+      <c r="F61" s="3" t="s">
         <v>107</v>
-      </c>
-      <c r="F61" s="3" t="s">
-        <v>109</v>
       </c>
     </row>
     <row r="62" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -2973,10 +2973,10 @@
         <v>71</v>
       </c>
       <c r="D62" t="s">
+        <v>106</v>
+      </c>
+      <c r="F62" s="3" t="s">
         <v>108</v>
-      </c>
-      <c r="F62" s="3" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
@@ -2984,13 +2984,13 @@
         <v>3</v>
       </c>
       <c r="D63" t="s">
+        <v>109</v>
+      </c>
+      <c r="E63" t="s">
+        <v>110</v>
+      </c>
+      <c r="F63" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="E63" t="s">
-        <v>112</v>
-      </c>
-      <c r="F63" s="3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
@@ -3004,10 +3004,10 @@
         <v>71</v>
       </c>
       <c r="D64" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F64" s="3" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
@@ -3021,10 +3021,10 @@
         <v>71</v>
       </c>
       <c r="D65" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F65" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
@@ -3038,10 +3038,10 @@
         <v>71</v>
       </c>
       <c r="D66" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F66" s="3" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
@@ -3055,10 +3055,10 @@
         <v>71</v>
       </c>
       <c r="D67" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F67" s="3" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
@@ -3072,10 +3072,10 @@
         <v>7</v>
       </c>
       <c r="D68" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F68" s="3" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
     </row>
     <row r="69" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
@@ -3089,10 +3089,10 @@
         <v>71</v>
       </c>
       <c r="D69" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F69" s="3" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
@@ -3100,13 +3100,13 @@
         <v>3</v>
       </c>
       <c r="D70" t="s">
+        <v>124</v>
+      </c>
+      <c r="E70" t="s">
+        <v>125</v>
+      </c>
+      <c r="F70" s="3" t="s">
         <v>126</v>
-      </c>
-      <c r="E70" t="s">
-        <v>127</v>
-      </c>
-      <c r="F70" s="3" t="s">
-        <v>128</v>
       </c>
     </row>
     <row r="71" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -3120,10 +3120,10 @@
         <v>71</v>
       </c>
       <c r="D71" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F71" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
@@ -3137,10 +3137,10 @@
         <v>71</v>
       </c>
       <c r="D72" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F72" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="73" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3154,10 +3154,10 @@
         <v>71</v>
       </c>
       <c r="D73" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F73" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="74" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3171,24 +3171,24 @@
         <v>71</v>
       </c>
       <c r="D74" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F74" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B75">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D75" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E75" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F75" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="76" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3202,10 +3202,10 @@
         <v>71</v>
       </c>
       <c r="D76" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F76" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
@@ -3219,10 +3219,10 @@
         <v>71</v>
       </c>
       <c r="D77" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F77" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="78" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3236,10 +3236,10 @@
         <v>71</v>
       </c>
       <c r="D78" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="F78" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
@@ -3247,13 +3247,13 @@
         <v>3</v>
       </c>
       <c r="D79" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E79" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="F79" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="80" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3267,10 +3267,10 @@
         <v>71</v>
       </c>
       <c r="D80" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="F80" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
     </row>
     <row r="81" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3284,10 +3284,10 @@
         <v>71</v>
       </c>
       <c r="D81" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="F81" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
     </row>
     <row r="82" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3301,10 +3301,10 @@
         <v>71</v>
       </c>
       <c r="D82" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="F82" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="83" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3318,24 +3318,24 @@
         <v>71</v>
       </c>
       <c r="D83" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="F83" s="3" t="s">
-        <v>403</v>
+        <v>399</v>
       </c>
     </row>
     <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="B84">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D84" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E84" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="F84" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="85" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
@@ -3349,10 +3349,10 @@
         <v>71</v>
       </c>
       <c r="D85" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>190</v>
+        <v>435</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">
@@ -3360,13 +3360,13 @@
         <v>3</v>
       </c>
       <c r="D86" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E86" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="F86" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="87" spans="1:6" ht="72" x14ac:dyDescent="0.3">
@@ -3380,10 +3380,10 @@
         <v>71</v>
       </c>
       <c r="D87" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="F87" s="3" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
     </row>
     <row r="88" spans="1:6" x14ac:dyDescent="0.3">
@@ -3391,13 +3391,13 @@
         <v>3</v>
       </c>
       <c r="D88" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E88" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="F88" s="3" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
     </row>
     <row r="89" spans="1:6" x14ac:dyDescent="0.3">
@@ -3411,10 +3411,10 @@
         <v>71</v>
       </c>
       <c r="D89" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="F89" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
     </row>
     <row r="90" spans="1:6" x14ac:dyDescent="0.3">
@@ -3428,10 +3428,10 @@
         <v>71</v>
       </c>
       <c r="D90" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="F90" s="3" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
     </row>
     <row r="91" spans="1:6" x14ac:dyDescent="0.3">
@@ -3439,10 +3439,10 @@
         <v>2</v>
       </c>
       <c r="D91" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="E91" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
     </row>
     <row r="92" spans="1:6" x14ac:dyDescent="0.3">
@@ -3450,10 +3450,10 @@
         <v>3</v>
       </c>
       <c r="D92" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E92" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
     </row>
     <row r="93" spans="1:6" x14ac:dyDescent="0.3">
@@ -3467,10 +3467,10 @@
         <v>71</v>
       </c>
       <c r="D93" t="s">
-        <v>195</v>
+        <v>192</v>
       </c>
       <c r="F93" s="3" t="s">
-        <v>194</v>
+        <v>191</v>
       </c>
     </row>
     <row r="94" spans="1:6" x14ac:dyDescent="0.3">
@@ -3484,10 +3484,10 @@
         <v>7</v>
       </c>
       <c r="D94" t="s">
-        <v>196</v>
+        <v>193</v>
       </c>
       <c r="F94" s="3" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="95" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -3501,10 +3501,10 @@
         <v>71</v>
       </c>
       <c r="D95" t="s">
-        <v>197</v>
+        <v>194</v>
       </c>
       <c r="F95" s="3" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
     </row>
     <row r="96" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3518,10 +3518,10 @@
         <v>71</v>
       </c>
       <c r="D96" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="F96" s="3" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
@@ -3535,10 +3535,10 @@
         <v>7</v>
       </c>
       <c r="D97" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="F97" s="3" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
@@ -3546,10 +3546,10 @@
         <v>3</v>
       </c>
       <c r="D98" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="E98" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
     </row>
     <row r="99" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3563,10 +3563,10 @@
         <v>71</v>
       </c>
       <c r="D99" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="F99" s="3" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
     </row>
     <row r="100" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3580,13 +3580,13 @@
         <v>71</v>
       </c>
       <c r="D100" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="E100" t="s">
-        <v>228</v>
+        <v>225</v>
       </c>
       <c r="F100" s="3" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
@@ -3600,10 +3600,10 @@
         <v>71</v>
       </c>
       <c r="D101" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="F101" s="3" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
     </row>
     <row r="102" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3617,10 +3617,10 @@
         <v>71</v>
       </c>
       <c r="D102" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F102" s="3" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
     </row>
     <row r="103" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3634,10 +3634,10 @@
         <v>71</v>
       </c>
       <c r="D103" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F103" s="3" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
@@ -3651,10 +3651,10 @@
         <v>71</v>
       </c>
       <c r="D104" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="F104" s="3" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
     </row>
     <row r="105" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3668,10 +3668,10 @@
         <v>71</v>
       </c>
       <c r="D105" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="F105" s="3" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
@@ -3685,10 +3685,10 @@
         <v>7</v>
       </c>
       <c r="D106" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F106" s="3" t="s">
-        <v>404</v>
+        <v>400</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -3702,10 +3702,10 @@
         <v>71</v>
       </c>
       <c r="D107" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="F107" s="3" t="s">
-        <v>405</v>
+        <v>401</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
@@ -3719,10 +3719,10 @@
         <v>71</v>
       </c>
       <c r="D108" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="F108" s="3" t="s">
-        <v>406</v>
+        <v>402</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
@@ -3736,10 +3736,10 @@
         <v>71</v>
       </c>
       <c r="D109" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="F109" s="3" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
@@ -3753,10 +3753,10 @@
         <v>71</v>
       </c>
       <c r="D110" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="F110" s="3" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
@@ -3770,10 +3770,10 @@
         <v>71</v>
       </c>
       <c r="D111" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="F111" s="3" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
@@ -3787,10 +3787,10 @@
         <v>71</v>
       </c>
       <c r="D112" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="F112" s="3" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
     </row>
     <row r="113" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3804,10 +3804,10 @@
         <v>71</v>
       </c>
       <c r="D113" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="F113" s="3" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
     </row>
     <row r="114" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3821,10 +3821,10 @@
         <v>71</v>
       </c>
       <c r="D114" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="F114" s="3" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
     </row>
     <row r="115" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -3838,10 +3838,10 @@
         <v>71</v>
       </c>
       <c r="D115" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="F115" s="3" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
@@ -3855,10 +3855,10 @@
         <v>71</v>
       </c>
       <c r="D116" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="F116" s="3" t="s">
-        <v>407</v>
+        <v>403</v>
       </c>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
@@ -3872,10 +3872,10 @@
         <v>71</v>
       </c>
       <c r="D117" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="F117" s="3" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
     </row>
     <row r="118" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3889,10 +3889,10 @@
         <v>71</v>
       </c>
       <c r="D118" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="F118" s="3" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
     </row>
     <row r="119" spans="1:6" x14ac:dyDescent="0.3">
@@ -3900,10 +3900,10 @@
         <v>3</v>
       </c>
       <c r="D119" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="E119" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
     </row>
     <row r="120" spans="1:6" ht="100.8" x14ac:dyDescent="0.3">
@@ -3917,10 +3917,10 @@
         <v>71</v>
       </c>
       <c r="D120" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="F120" s="3" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
     </row>
     <row r="121" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3934,10 +3934,10 @@
         <v>71</v>
       </c>
       <c r="D121" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="F121" s="3" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
@@ -3945,10 +3945,10 @@
         <v>3</v>
       </c>
       <c r="D122" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="E122" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
     </row>
     <row r="123" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3962,10 +3962,10 @@
         <v>71</v>
       </c>
       <c r="D123" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F123" s="3" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
@@ -3979,13 +3979,13 @@
         <v>71</v>
       </c>
       <c r="D124" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="E124" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="F124" s="3" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
@@ -3999,10 +3999,10 @@
         <v>71</v>
       </c>
       <c r="D125" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="F125" s="3" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
@@ -4016,10 +4016,10 @@
         <v>71</v>
       </c>
       <c r="D126" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="F126" s="3" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
     </row>
     <row r="127" spans="1:6" ht="201.6" x14ac:dyDescent="0.3">
@@ -4033,10 +4033,10 @@
         <v>71</v>
       </c>
       <c r="D127" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="F127" s="3" t="s">
-        <v>408</v>
+        <v>404</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
@@ -4044,10 +4044,10 @@
         <v>3</v>
       </c>
       <c r="D128" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="E128" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="129" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
@@ -4061,10 +4061,10 @@
         <v>71</v>
       </c>
       <c r="D129" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="F129" s="3" t="s">
-        <v>409</v>
+        <v>405</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
@@ -4072,10 +4072,10 @@
         <v>2</v>
       </c>
       <c r="D130" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="E130" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
     </row>
     <row r="131" spans="1:6" x14ac:dyDescent="0.3">
@@ -4083,10 +4083,10 @@
         <v>3</v>
       </c>
       <c r="D131" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="E131" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
     </row>
     <row r="132" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4100,10 +4100,10 @@
         <v>71</v>
       </c>
       <c r="D132" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="F132" s="3" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
     </row>
     <row r="133" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4117,10 +4117,10 @@
         <v>71</v>
       </c>
       <c r="D133" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="F133" s="3" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
@@ -4134,10 +4134,10 @@
         <v>71</v>
       </c>
       <c r="D134" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="F134" s="3" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
@@ -4145,10 +4145,10 @@
         <v>3</v>
       </c>
       <c r="D135" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="E135" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
     </row>
     <row r="136" spans="1:6" ht="86.4" x14ac:dyDescent="0.3">
@@ -4162,10 +4162,10 @@
         <v>71</v>
       </c>
       <c r="D136" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="F136" s="3" t="s">
-        <v>410</v>
+        <v>406</v>
       </c>
     </row>
     <row r="137" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -4179,10 +4179,10 @@
         <v>71</v>
       </c>
       <c r="D137" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="F137" s="3" t="s">
-        <v>411</v>
+        <v>407</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
@@ -4190,10 +4190,10 @@
         <v>3</v>
       </c>
       <c r="D138" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="E138" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
     </row>
     <row r="139" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
@@ -4207,10 +4207,10 @@
         <v>71</v>
       </c>
       <c r="D139" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="F139" s="3" t="s">
-        <v>412</v>
+        <v>408</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
@@ -4218,10 +4218,10 @@
         <v>3</v>
       </c>
       <c r="D140" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="E140" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
     </row>
     <row r="141" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
@@ -4235,10 +4235,10 @@
         <v>71</v>
       </c>
       <c r="D141" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="F141" s="3" t="s">
-        <v>413</v>
+        <v>409</v>
       </c>
     </row>
     <row r="142" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
@@ -4252,10 +4252,10 @@
         <v>71</v>
       </c>
       <c r="D142" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="F142" s="3" t="s">
-        <v>414</v>
+        <v>410</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
@@ -4263,10 +4263,10 @@
         <v>3</v>
       </c>
       <c r="D143" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="E143" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
@@ -4280,10 +4280,10 @@
         <v>71</v>
       </c>
       <c r="D144" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="F144" s="3" t="s">
-        <v>415</v>
+        <v>411</v>
       </c>
     </row>
     <row r="145" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4297,10 +4297,10 @@
         <v>7</v>
       </c>
       <c r="D145" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="F145" s="3" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
     </row>
     <row r="146" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4314,10 +4314,10 @@
         <v>71</v>
       </c>
       <c r="D146" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F146" s="3" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
     </row>
     <row r="147" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4331,10 +4331,10 @@
         <v>71</v>
       </c>
       <c r="D147" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="F147" s="3" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
     </row>
     <row r="148" spans="1:6" ht="57.6" x14ac:dyDescent="0.3">
@@ -4348,10 +4348,10 @@
         <v>71</v>
       </c>
       <c r="D148" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="F148" s="3" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
     </row>
     <row r="149" spans="1:6" x14ac:dyDescent="0.3">
@@ -4359,10 +4359,10 @@
         <v>3</v>
       </c>
       <c r="D149" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="E149" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
     </row>
     <row r="150" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4376,10 +4376,10 @@
         <v>71</v>
       </c>
       <c r="D150" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="F150" s="3" t="s">
-        <v>416</v>
+        <v>412</v>
       </c>
     </row>
     <row r="151" spans="1:6" ht="115.2" x14ac:dyDescent="0.3">
@@ -4393,10 +4393,10 @@
         <v>71</v>
       </c>
       <c r="D151" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="F151" s="3" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
     </row>
     <row r="152" spans="1:6" ht="72" x14ac:dyDescent="0.3">
@@ -4410,10 +4410,10 @@
         <v>7</v>
       </c>
       <c r="D152" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="F152" s="3" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
     </row>
     <row r="153" spans="1:6" x14ac:dyDescent="0.3">
@@ -4421,10 +4421,10 @@
         <v>2</v>
       </c>
       <c r="D153" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="E153" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
     </row>
     <row r="154" spans="1:6" ht="158.4" x14ac:dyDescent="0.3">
@@ -4438,10 +4438,10 @@
         <v>7</v>
       </c>
       <c r="D154" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="F154" s="3" t="s">
-        <v>417</v>
+        <v>413</v>
       </c>
     </row>
     <row r="155" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4455,10 +4455,10 @@
         <v>71</v>
       </c>
       <c r="D155" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F155" s="3" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="156" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -4472,10 +4472,10 @@
         <v>7</v>
       </c>
       <c r="D156" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="F156" s="3" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
     </row>
     <row r="157" spans="1:6" x14ac:dyDescent="0.3">
@@ -4483,10 +4483,10 @@
         <v>2</v>
       </c>
       <c r="D157" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="E157" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
     </row>
     <row r="158" spans="1:6" x14ac:dyDescent="0.3">
@@ -4500,10 +4500,10 @@
         <v>71</v>
       </c>
       <c r="D158" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="F158" s="3" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
     </row>
     <row r="159" spans="1:6" x14ac:dyDescent="0.3">
@@ -4511,13 +4511,13 @@
         <v>3</v>
       </c>
       <c r="D159" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="E159" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F159" s="3" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="160" spans="1:6" x14ac:dyDescent="0.3">
@@ -4531,10 +4531,10 @@
         <v>71</v>
       </c>
       <c r="D160" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="F160" s="3" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
@@ -4548,10 +4548,10 @@
         <v>71</v>
       </c>
       <c r="D161" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="F161" s="3" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
@@ -4565,10 +4565,10 @@
         <v>71</v>
       </c>
       <c r="D162" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="F162" s="3" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
     </row>
     <row r="163" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4582,10 +4582,10 @@
         <v>71</v>
       </c>
       <c r="D163" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="F163" s="3" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
@@ -4593,13 +4593,13 @@
         <v>3</v>
       </c>
       <c r="D164" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="E164" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="F164" s="3" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
@@ -4613,10 +4613,10 @@
         <v>71</v>
       </c>
       <c r="D165" t="s">
+        <v>324</v>
+      </c>
+      <c r="F165" s="3" t="s">
         <v>327</v>
-      </c>
-      <c r="F165" s="3" t="s">
-        <v>330</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
@@ -4630,10 +4630,10 @@
         <v>71</v>
       </c>
       <c r="D166" t="s">
+        <v>325</v>
+      </c>
+      <c r="F166" s="3" t="s">
         <v>328</v>
-      </c>
-      <c r="F166" s="3" t="s">
-        <v>331</v>
       </c>
     </row>
     <row r="167" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4647,10 +4647,10 @@
         <v>71</v>
       </c>
       <c r="D167" t="s">
+        <v>326</v>
+      </c>
+      <c r="F167" s="3" t="s">
         <v>329</v>
-      </c>
-      <c r="F167" s="3" t="s">
-        <v>332</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
@@ -4658,10 +4658,10 @@
         <v>3</v>
       </c>
       <c r="D168" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="E168" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
@@ -4675,10 +4675,10 @@
         <v>71</v>
       </c>
       <c r="D169" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="F169" s="3" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
@@ -4692,13 +4692,13 @@
         <v>71</v>
       </c>
       <c r="D170" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="E170" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="F170" s="3" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
     </row>
     <row r="171" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4712,10 +4712,10 @@
         <v>71</v>
       </c>
       <c r="D171" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="F171" s="3" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
     </row>
     <row r="172" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4729,10 +4729,10 @@
         <v>71</v>
       </c>
       <c r="D172" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="F172" s="3" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
     </row>
     <row r="173" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -4746,10 +4746,10 @@
         <v>71</v>
       </c>
       <c r="D173" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F173" s="3" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
     </row>
     <row r="174" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4763,10 +4763,10 @@
         <v>71</v>
       </c>
       <c r="D174" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="F174" s="3" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
     </row>
     <row r="175" spans="1:6" x14ac:dyDescent="0.3">
@@ -4774,13 +4774,13 @@
         <v>3</v>
       </c>
       <c r="D175" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="E175" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="F175" s="3" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
     </row>
     <row r="176" spans="1:6" x14ac:dyDescent="0.3">
@@ -4794,10 +4794,10 @@
         <v>71</v>
       </c>
       <c r="D176" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="F176" s="3" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="177" spans="1:6" x14ac:dyDescent="0.3">
@@ -4811,10 +4811,10 @@
         <v>71</v>
       </c>
       <c r="D177" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="F177" s="3" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
     </row>
     <row r="178" spans="1:6" x14ac:dyDescent="0.3">
@@ -4828,10 +4828,10 @@
         <v>71</v>
       </c>
       <c r="D178" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="F178" s="3" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
     </row>
     <row r="179" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4845,10 +4845,10 @@
         <v>71</v>
       </c>
       <c r="D179" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="F179" s="3" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
     </row>
     <row r="180" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4862,10 +4862,10 @@
         <v>71</v>
       </c>
       <c r="D180" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="F180" s="3" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="181" spans="1:6" x14ac:dyDescent="0.3">
@@ -4879,10 +4879,10 @@
         <v>71</v>
       </c>
       <c r="D181" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="F181" s="3" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
     </row>
     <row r="182" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4896,10 +4896,10 @@
         <v>71</v>
       </c>
       <c r="D182" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="F182" s="3" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
     </row>
     <row r="183" spans="1:6" ht="43.2" x14ac:dyDescent="0.3">
@@ -4913,10 +4913,10 @@
         <v>71</v>
       </c>
       <c r="D183" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="F183" s="3" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="184" spans="1:6" x14ac:dyDescent="0.3">
@@ -4930,10 +4930,10 @@
         <v>71</v>
       </c>
       <c r="D184" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="F184" s="3" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
     </row>
     <row r="185" spans="1:6" x14ac:dyDescent="0.3">
@@ -4947,10 +4947,10 @@
         <v>71</v>
       </c>
       <c r="D185" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F185" s="3" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
     </row>
     <row r="186" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4964,10 +4964,10 @@
         <v>71</v>
       </c>
       <c r="D186" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
       <c r="F186" s="3" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
     </row>
     <row r="187" spans="1:6" x14ac:dyDescent="0.3">
@@ -4981,10 +4981,10 @@
         <v>71</v>
       </c>
       <c r="D187" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="F187" s="3" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="188" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -4998,10 +4998,10 @@
         <v>71</v>
       </c>
       <c r="D188" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F188" s="3" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="189" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -5015,10 +5015,10 @@
         <v>71</v>
       </c>
       <c r="D189" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="F189" s="3" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="190" spans="1:6" x14ac:dyDescent="0.3">
@@ -5026,13 +5026,13 @@
         <v>3</v>
       </c>
       <c r="D190" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="E190" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="F190" s="3" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="191" spans="1:6" x14ac:dyDescent="0.3">
@@ -5046,10 +5046,10 @@
         <v>71</v>
       </c>
       <c r="D191" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="F191" s="3" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
     </row>
     <row r="192" spans="1:6" x14ac:dyDescent="0.3">
@@ -5063,10 +5063,10 @@
         <v>71</v>
       </c>
       <c r="D192" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="F192" s="3" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="193" spans="1:6" x14ac:dyDescent="0.3">
@@ -5074,10 +5074,10 @@
         <v>2</v>
       </c>
       <c r="D193" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="E193" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="194" spans="1:6" ht="72" x14ac:dyDescent="0.3">
@@ -5091,10 +5091,10 @@
         <v>71</v>
       </c>
       <c r="D194" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="F194" s="3" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
     </row>
     <row r="195" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -5108,10 +5108,10 @@
         <v>71</v>
       </c>
       <c r="D195" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="F195" s="3" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="196" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -5125,10 +5125,10 @@
         <v>71</v>
       </c>
       <c r="D196" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="F196" s="3" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
     </row>
     <row r="197" spans="1:6" ht="72" x14ac:dyDescent="0.3">
@@ -5142,10 +5142,10 @@
         <v>7</v>
       </c>
       <c r="D197" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="F197" s="3" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
   </sheetData>
@@ -5162,7 +5162,7 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>418</v>
+        <v>414</v>
       </c>
       <c r="B1" t="s">
         <v>6</v>
@@ -5173,7 +5173,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="s">
-        <v>429</v>
+        <v>425</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correction coquille ISO 19011
</commit_message>
<xml_diff>
--- a/tools/excel/PASSI/PASSI.xlsx
+++ b/tools/excel/PASSI/PASSI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cintamaya-my.sharepoint.com/personal/arthur_lafont_cintamaya_com/Documents/02.Cinta/Ciso import tool/ciso-assistant-community/tools/excel/PASSI/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="13_ncr:1_{C69144C6-7723-45D0-AD2A-8B323A6D48CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{827C76A5-B2E3-40AB-B035-53C2628F1EEC}"/>
+  <xr:revisionPtr revIDLastSave="92" documentId="13_ncr:1_{C69144C6-7723-45D0-AD2A-8B323A6D48CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{75E1B634-E0F5-493C-8258-D294B9B8730D}"/>
   <bookViews>
     <workbookView xWindow="14205" yWindow="-16425" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1417,16 +1417,16 @@
     <t>Il est recommandé que le prestataire mette en œuvre la démarche décrite dans le guide pour homologuer son système d’information.</t>
   </si>
   <si>
-    <t>Les auditeurs et responsables d’équipe doivent maîtriser les bonnes pratiques et la méthodologie d’audit décrites dans la norme  ISO 1901.</t>
-  </si>
-  <si>
-    <t>Les auditeurs doivent posséder les qualités personnelles décrites au chapitre « 7.2.2 Comportements personnels » de la norme  ISO 1901.</t>
-  </si>
-  <si>
     <t>préciser que le prestataire peut incorporer dans l’équipe d’audit un ou plusieurs experts pour participer à la réalisation de certaines activités d’audit lorsque ces dernières requièrent des connaissances ou des compétences spécifiques dont les auditeurs ne disposent pas sous réserve que : 
 i. il existe un cadre contractuel entre le prestataire et les experts ;
 ii. le recours aux experts est accepté par le commanditaire ;
 iii. les experts sont dûment encadrés par le responsable d’équipe.</t>
+  </si>
+  <si>
+    <t>Les auditeurs et responsables d’équipe doivent maîtriser les bonnes pratiques et la méthodologie d’audit décrites dans la norme  ISO 19011.</t>
+  </si>
+  <si>
+    <t>Les auditeurs doivent posséder les qualités personnelles décrites au chapitre « 7.2.2 Comportements personnels » de la norme  ISO 19011.</t>
   </si>
 </sst>
 </file>
@@ -2641,7 +2641,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="41" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>3</v>
       </c>
@@ -2655,10 +2655,10 @@
         <v>81</v>
       </c>
       <c r="F41" s="3" t="s">
-        <v>433</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
+        <v>434</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>3</v>
       </c>
@@ -2672,7 +2672,7 @@
         <v>82</v>
       </c>
       <c r="F42" s="8" t="s">
-        <v>434</v>
+        <v>435</v>
       </c>
     </row>
     <row r="43" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
@@ -3352,7 +3352,7 @@
         <v>154</v>
       </c>
       <c r="F85" s="3" t="s">
-        <v>435</v>
+        <v>433</v>
       </c>
     </row>
     <row r="86" spans="1:6" x14ac:dyDescent="0.3">

</xml_diff>